<commit_message>
optimize project list and capacity scheduling
</commit_message>
<xml_diff>
--- a/templates/人员资料导入模板.xlsx
+++ b/templates/人员资料导入模板.xlsx
@@ -411,7 +411,7 @@
     <col min="6" max="6" width="22.83203125" customWidth="1"/>
     <col min="7" max="7" width="26.83203125" customWidth="1"/>
     <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
     <col min="10" max="10" width="12.83203125" customWidth="1"/>
     <col min="11" max="11" width="16.83203125" customWidth="1"/>
     <col min="12" max="12" width="12.83203125" customWidth="1"/>
@@ -444,7 +444,7 @@
         <v>标准总产能</v>
       </c>
       <c r="I1" t="str">
-        <v>产能释放日期</v>
+        <v>预计产能释放日期</v>
       </c>
       <c r="J1" t="str">
         <v>在岗状态</v>
@@ -549,10 +549,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>产能释放日期</v>
+        <v>预计产能释放日期</v>
       </c>
       <c r="B10" t="str">
-        <v>日期未到前，该人员不会进入可调度名单。</v>
+        <v>选填，仅用于排期参考；商务、PM 等持续性岗位或暂无明确日期时可留空。可安排与否按全部有效项目的产能占用合计判断。</v>
       </c>
     </row>
     <row r="11">

</xml_diff>